<commit_message>
modified:   recomendador/Tabla_Maestra_ZKTeco.xlsx 	modified:   recomendador/catalogo_zkteco.json 	new file:   recomendador/img/ZKT0810089.png 	new file:   recomendador/img/ZKT1140003.png 	new file:   recomendador/img/icons/favicon.png 	modified:   recomendador/index.html
</commit_message>
<xml_diff>
--- a/recomendador/Tabla_Maestra_ZKTeco.xlsx
+++ b/recomendador/Tabla_Maestra_ZKTeco.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TVCMTY-57298\Documents\recomendador\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1B203C5-7C64-4E26-BD57-DB42F1DDFE8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{222444EE-EB6D-484E-B502-BA2B6D796D3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="704" xr2:uid="{DB513028-4120-4D60-A8C2-889CF1E9B842}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="704" activeTab="4" xr2:uid="{DB513028-4120-4D60-A8C2-889CF1E9B842}"/>
   </bookViews>
   <sheets>
     <sheet name="Equipos" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3201" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3301" uniqueCount="287">
   <si>
     <t>ID</t>
   </si>
@@ -883,6 +883,33 @@
     <t>Módulo DM-10 por RS485; 
 Lector RS485 como FR1200 o FR1500 (solo RFID); 
 Lector Wiegand como KR500 o alguna UHF por medio de WR485.</t>
+  </si>
+  <si>
+    <t>ZKT0810089</t>
+  </si>
+  <si>
+    <t>Horus H1</t>
+  </si>
+  <si>
+    <t>5,200 mAh</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/75230</t>
+  </si>
+  <si>
+    <t>5 horas</t>
+  </si>
+  <si>
+    <t>ZKT1140003</t>
+  </si>
+  <si>
+    <t>D3</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/88760</t>
   </si>
 </sst>
 </file>
@@ -932,7 +959,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -957,6 +984,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1272,7 +1302,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92ADD60D-2C97-426D-9463-37EADD9F0616}">
-  <dimension ref="A1:AB51"/>
+  <dimension ref="A1:AB53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="20" bestFit="1" customWidth="1"/>
@@ -1283,7 +1313,8 @@
     <col min="16" max="17" width="11.5546875" style="5"/>
     <col min="18" max="18" width="15.109375" style="5" customWidth="1"/>
     <col min="19" max="19" width="16.44140625" customWidth="1"/>
-    <col min="20" max="21" width="17.44140625" customWidth="1"/>
+    <col min="20" max="20" width="17.44140625" customWidth="1"/>
+    <col min="21" max="21" width="17.44140625" style="7" customWidth="1"/>
     <col min="22" max="22" width="23" customWidth="1"/>
     <col min="23" max="23" width="25" customWidth="1"/>
     <col min="24" max="24" width="17.44140625" customWidth="1"/>
@@ -5189,6 +5220,154 @@
         <v>275</v>
       </c>
     </row>
+    <row r="52" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A52" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="E52" s="5">
+        <v>50000</v>
+      </c>
+      <c r="F52" s="5">
+        <v>50000</v>
+      </c>
+      <c r="G52" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H52" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I52" s="5">
+        <v>50000</v>
+      </c>
+      <c r="J52" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="K52" s="5">
+        <v>50000</v>
+      </c>
+      <c r="L52" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="M52" s="5">
+        <v>1000000</v>
+      </c>
+      <c r="N52" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="O52" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="P52" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q52" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="R52" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="U52" s="8" t="s">
+        <v>267</v>
+      </c>
+      <c r="X52" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="Y52" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="Z52" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="AA52" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="AB52" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="53" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A53" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="E53" s="5">
+        <v>1000</v>
+      </c>
+      <c r="F53" s="5">
+        <v>500</v>
+      </c>
+      <c r="G53" s="5">
+        <v>1000</v>
+      </c>
+      <c r="H53" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I53" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="J53" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K53" s="5">
+        <v>1000</v>
+      </c>
+      <c r="L53" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="M53" s="5">
+        <v>150000</v>
+      </c>
+      <c r="N53" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="O53" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="P53" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q53" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="R53" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="U53" s="7" t="s">
+        <v>268</v>
+      </c>
+      <c r="X53" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y53" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Z53" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="AA53" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="AB53" t="s">
+        <v>286</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5198,10 +5377,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BD560C2-BF1C-4DA5-BB4B-058D0BDCFFDC}">
-  <dimension ref="A1:M51"/>
+  <dimension ref="A1:M53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="18.21875" customWidth="1"/>
+    <col min="3" max="3" width="18.21875" style="9" customWidth="1"/>
     <col min="5" max="5" width="14.5546875" customWidth="1"/>
     <col min="6" max="6" width="14.21875" customWidth="1"/>
     <col min="7" max="7" width="14.33203125" customWidth="1"/>
@@ -7184,6 +7363,82 @@
         <v>277</v>
       </c>
     </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A52" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C52" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G52" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H52" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I52" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J52" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="K52" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="L52" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A53" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C53" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G53" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H53" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I53" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J53" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="K53" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="L53" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -7192,7 +7447,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01D188FE-0A5F-4722-9988-1447CAAEAEC2}">
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
@@ -7625,7 +7880,7 @@
         <v>23</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>44</v>
@@ -7648,7 +7903,7 @@
         <v>23</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>44</v>
@@ -7671,7 +7926,7 @@
         <v>20</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>44</v>
@@ -7694,7 +7949,7 @@
         <v>23</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>44</v>
@@ -8371,6 +8626,52 @@
       </c>
       <c r="G51" s="3" t="s">
         <v>43</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A52" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F52" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G52" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A53" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F53" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G53" s="3" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -8548,7 +8849,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFD578E9-46E5-410E-B6CF-C9D9B5BCC9DE}">
-  <dimension ref="A1:L205"/>
+  <dimension ref="A1:L209"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="17.109375" customWidth="1"/>
@@ -10574,39 +10875,39 @@
         <v>142</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C98" s="3" t="s">
         <v>38</v>
       </c>
       <c r="D98" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E98" s="3" t="s">
         <v>57</v>
       </c>
       <c r="F98" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" s="4" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D99" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E99" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F99" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
@@ -10614,7 +10915,7 @@
         <v>147</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C100" s="3" t="s">
         <v>37</v>
@@ -10634,7 +10935,7 @@
         <v>147</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C101" s="3" t="s">
         <v>37</v>
@@ -10643,7 +10944,7 @@
         <v>43</v>
       </c>
       <c r="E101" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F101" s="3" t="s">
         <v>21</v>
@@ -10654,19 +10955,19 @@
         <v>147</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C102" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D102" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E102" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F102" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
@@ -10674,19 +10975,19 @@
         <v>147</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C103" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D103" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E103" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F103" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
@@ -10694,30 +10995,30 @@
         <v>147</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C104" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D104" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E104" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F104" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105" s="4" t="s">
-        <v>147</v>
+        <v>233</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D105" s="3" t="s">
         <v>44</v>
@@ -10734,7 +11035,7 @@
         <v>233</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C106" s="3" t="s">
         <v>39</v>
@@ -10750,11 +11051,11 @@
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A107" s="4" t="s">
-        <v>233</v>
+      <c r="A107" t="s">
+        <v>236</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C107" s="3" t="s">
         <v>39</v>
@@ -10774,7 +11075,7 @@
         <v>236</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C108" s="3" t="s">
         <v>39</v>
@@ -10790,11 +11091,11 @@
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A109" t="s">
-        <v>236</v>
+      <c r="A109" s="4" t="s">
+        <v>239</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C109" s="3" t="s">
         <v>39</v>
@@ -10814,7 +11115,7 @@
         <v>239</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C110" s="3" t="s">
         <v>39</v>
@@ -10831,22 +11132,22 @@
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" s="4" t="s">
-        <v>239</v>
+        <v>158</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D111" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E111" s="3" t="s">
         <v>52</v>
       </c>
       <c r="F111" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
@@ -10854,7 +11155,7 @@
         <v>158</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C112" s="3" t="s">
         <v>37</v>
@@ -10874,7 +11175,7 @@
         <v>158</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C113" s="3" t="s">
         <v>37</v>
@@ -10883,7 +11184,7 @@
         <v>43</v>
       </c>
       <c r="E113" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F113" s="3" t="s">
         <v>21</v>
@@ -10894,7 +11195,7 @@
         <v>158</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C114" s="3" t="s">
         <v>37</v>
@@ -10911,10 +11212,10 @@
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115" s="4" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="C115" s="3" t="s">
         <v>37</v>
@@ -10923,7 +11224,7 @@
         <v>43</v>
       </c>
       <c r="E115" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F115" s="3" t="s">
         <v>21</v>
@@ -10934,7 +11235,7 @@
         <v>162</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C116" s="3" t="s">
         <v>37</v>
@@ -10954,7 +11255,7 @@
         <v>162</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C117" s="3" t="s">
         <v>37</v>
@@ -10963,7 +11264,7 @@
         <v>43</v>
       </c>
       <c r="E117" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F117" s="3" t="s">
         <v>21</v>
@@ -10974,7 +11275,7 @@
         <v>162</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C118" s="3" t="s">
         <v>37</v>
@@ -10990,23 +11291,23 @@
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A119" s="4" t="s">
-        <v>162</v>
+      <c r="A119">
+        <v>75019</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C119" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D119" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E119" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F119" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.3">
@@ -11014,7 +11315,7 @@
         <v>75019</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C120" s="3" t="s">
         <v>37</v>
@@ -11030,14 +11331,14 @@
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A121">
-        <v>75019</v>
+      <c r="A121" s="4" t="s">
+        <v>173</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C121" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D121" s="3" t="s">
         <v>44</v>
@@ -11054,7 +11355,7 @@
         <v>173</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C122" s="3" t="s">
         <v>39</v>
@@ -11071,13 +11372,13 @@
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A123" s="4" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C123" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D123" s="3" t="s">
         <v>44</v>
@@ -11094,7 +11395,7 @@
         <v>176</v>
       </c>
       <c r="B124" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C124" s="3" t="s">
         <v>37</v>
@@ -11111,22 +11412,22 @@
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A125" s="4" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="B125" s="3" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="C125" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D125" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E125" s="3" t="s">
         <v>52</v>
       </c>
       <c r="F125" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.3">
@@ -11134,7 +11435,7 @@
         <v>183</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C126" s="3" t="s">
         <v>37</v>
@@ -11154,7 +11455,7 @@
         <v>183</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C127" s="3" t="s">
         <v>37</v>
@@ -11163,7 +11464,7 @@
         <v>43</v>
       </c>
       <c r="E127" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F127" s="3" t="s">
         <v>21</v>
@@ -11174,19 +11475,19 @@
         <v>183</v>
       </c>
       <c r="B128" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C128" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D128" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E128" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F128" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.3">
@@ -11194,19 +11495,19 @@
         <v>183</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C129" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D129" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E129" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F129" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.3">
@@ -11214,39 +11515,39 @@
         <v>183</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C130" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D130" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E130" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F130" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A131" s="4" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B131" s="3" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="C131" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D131" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E131" s="3" t="s">
         <v>52</v>
       </c>
       <c r="F131" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.3">
@@ -11254,7 +11555,7 @@
         <v>186</v>
       </c>
       <c r="B132" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C132" s="3" t="s">
         <v>37</v>
@@ -11274,7 +11575,7 @@
         <v>186</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C133" s="3" t="s">
         <v>37</v>
@@ -11283,7 +11584,7 @@
         <v>43</v>
       </c>
       <c r="E133" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F133" s="3" t="s">
         <v>21</v>
@@ -11294,19 +11595,19 @@
         <v>186</v>
       </c>
       <c r="B134" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C134" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D134" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E134" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F134" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.3">
@@ -11314,19 +11615,19 @@
         <v>186</v>
       </c>
       <c r="B135" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C135" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D135" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E135" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F135" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.3">
@@ -11334,39 +11635,39 @@
         <v>186</v>
       </c>
       <c r="B136" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C136" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D136" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E136" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F136" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A137" s="4" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B137" s="3" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="C137" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D137" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E137" s="3" t="s">
         <v>52</v>
       </c>
       <c r="F137" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.3">
@@ -11374,7 +11675,7 @@
         <v>189</v>
       </c>
       <c r="B138" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C138" s="3" t="s">
         <v>37</v>
@@ -11394,7 +11695,7 @@
         <v>189</v>
       </c>
       <c r="B139" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C139" s="3" t="s">
         <v>37</v>
@@ -11403,7 +11704,7 @@
         <v>43</v>
       </c>
       <c r="E139" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F139" s="3" t="s">
         <v>21</v>
@@ -11414,19 +11715,19 @@
         <v>189</v>
       </c>
       <c r="B140" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C140" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D140" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E140" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F140" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.3">
@@ -11434,19 +11735,19 @@
         <v>189</v>
       </c>
       <c r="B141" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C141" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D141" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E141" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F141" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.3">
@@ -11454,39 +11755,39 @@
         <v>189</v>
       </c>
       <c r="B142" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C142" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D142" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E142" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F142" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A143" s="4" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B143" s="3" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="C143" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D143" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E143" s="3" t="s">
         <v>52</v>
       </c>
       <c r="F143" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.3">
@@ -11494,7 +11795,7 @@
         <v>192</v>
       </c>
       <c r="B144" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C144" s="3" t="s">
         <v>37</v>
@@ -11514,7 +11815,7 @@
         <v>192</v>
       </c>
       <c r="B145" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C145" s="3" t="s">
         <v>37</v>
@@ -11523,7 +11824,7 @@
         <v>43</v>
       </c>
       <c r="E145" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F145" s="3" t="s">
         <v>21</v>
@@ -11534,19 +11835,19 @@
         <v>192</v>
       </c>
       <c r="B146" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C146" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D146" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E146" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F146" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.3">
@@ -11554,19 +11855,19 @@
         <v>192</v>
       </c>
       <c r="B147" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C147" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D147" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E147" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F147" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.3">
@@ -11574,39 +11875,39 @@
         <v>192</v>
       </c>
       <c r="B148" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C148" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D148" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E148" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F148" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A149" s="4" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="B149" s="3" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="C149" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D149" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E149" s="3" t="s">
         <v>52</v>
       </c>
       <c r="F149" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.3">
@@ -11614,7 +11915,7 @@
         <v>196</v>
       </c>
       <c r="B150" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C150" s="3" t="s">
         <v>37</v>
@@ -11634,7 +11935,7 @@
         <v>196</v>
       </c>
       <c r="B151" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C151" s="3" t="s">
         <v>37</v>
@@ -11643,7 +11944,7 @@
         <v>43</v>
       </c>
       <c r="E151" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F151" s="3" t="s">
         <v>21</v>
@@ -11654,19 +11955,19 @@
         <v>196</v>
       </c>
       <c r="B152" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C152" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D152" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E152" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F152" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.3">
@@ -11674,19 +11975,19 @@
         <v>196</v>
       </c>
       <c r="B153" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C153" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D153" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E153" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F153" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.3">
@@ -11694,39 +11995,39 @@
         <v>196</v>
       </c>
       <c r="B154" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C154" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D154" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E154" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F154" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A155" s="4" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="B155" s="3" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="C155" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D155" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E155" s="3" t="s">
         <v>52</v>
       </c>
       <c r="F155" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.3">
@@ -11734,7 +12035,7 @@
         <v>200</v>
       </c>
       <c r="B156" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C156" s="3" t="s">
         <v>37</v>
@@ -11754,7 +12055,7 @@
         <v>200</v>
       </c>
       <c r="B157" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C157" s="3" t="s">
         <v>37</v>
@@ -11763,7 +12064,7 @@
         <v>43</v>
       </c>
       <c r="E157" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F157" s="3" t="s">
         <v>21</v>
@@ -11774,19 +12075,19 @@
         <v>200</v>
       </c>
       <c r="B158" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C158" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D158" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E158" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F158" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.3">
@@ -11794,19 +12095,19 @@
         <v>200</v>
       </c>
       <c r="B159" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C159" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D159" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E159" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F159" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.3">
@@ -11814,39 +12115,39 @@
         <v>200</v>
       </c>
       <c r="B160" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C160" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D160" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E160" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F160" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A161" s="4" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="B161" s="3" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="C161" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D161" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E161" s="3" t="s">
         <v>52</v>
       </c>
       <c r="F161" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.3">
@@ -11854,7 +12155,7 @@
         <v>203</v>
       </c>
       <c r="B162" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C162" s="3" t="s">
         <v>37</v>
@@ -11874,7 +12175,7 @@
         <v>203</v>
       </c>
       <c r="B163" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C163" s="3" t="s">
         <v>37</v>
@@ -11883,7 +12184,7 @@
         <v>43</v>
       </c>
       <c r="E163" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F163" s="3" t="s">
         <v>21</v>
@@ -11894,7 +12195,7 @@
         <v>203</v>
       </c>
       <c r="B164" s="3" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C164" s="3" t="s">
         <v>37</v>
@@ -11911,10 +12212,10 @@
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A165" s="4" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="B165" s="3" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="C165" s="3" t="s">
         <v>37</v>
@@ -11923,7 +12224,7 @@
         <v>43</v>
       </c>
       <c r="E165" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F165" s="3" t="s">
         <v>21</v>
@@ -11934,7 +12235,7 @@
         <v>209</v>
       </c>
       <c r="B166" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C166" s="3" t="s">
         <v>37</v>
@@ -11954,7 +12255,7 @@
         <v>209</v>
       </c>
       <c r="B167" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C167" s="3" t="s">
         <v>37</v>
@@ -11963,7 +12264,7 @@
         <v>43</v>
       </c>
       <c r="E167" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F167" s="3" t="s">
         <v>21</v>
@@ -11974,19 +12275,19 @@
         <v>209</v>
       </c>
       <c r="B168" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C168" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D168" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E168" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F168" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="169" spans="1:6" x14ac:dyDescent="0.3">
@@ -11994,19 +12295,19 @@
         <v>209</v>
       </c>
       <c r="B169" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C169" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D169" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E169" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F169" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="170" spans="1:6" x14ac:dyDescent="0.3">
@@ -12014,39 +12315,39 @@
         <v>209</v>
       </c>
       <c r="B170" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C170" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D170" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E170" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F170" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A171" s="4" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B171" s="3" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="C171" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D171" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E171" s="3" t="s">
         <v>52</v>
       </c>
       <c r="F171" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.3">
@@ -12054,7 +12355,7 @@
         <v>212</v>
       </c>
       <c r="B172" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C172" s="3" t="s">
         <v>37</v>
@@ -12074,7 +12375,7 @@
         <v>212</v>
       </c>
       <c r="B173" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C173" s="3" t="s">
         <v>37</v>
@@ -12083,7 +12384,7 @@
         <v>43</v>
       </c>
       <c r="E173" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F173" s="3" t="s">
         <v>21</v>
@@ -12094,19 +12395,19 @@
         <v>212</v>
       </c>
       <c r="B174" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C174" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D174" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E174" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F174" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="175" spans="1:6" x14ac:dyDescent="0.3">
@@ -12114,19 +12415,19 @@
         <v>212</v>
       </c>
       <c r="B175" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C175" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D175" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E175" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F175" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="176" spans="1:6" x14ac:dyDescent="0.3">
@@ -12134,39 +12435,39 @@
         <v>212</v>
       </c>
       <c r="B176" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C176" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D176" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E176" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F176" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="177" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A177" s="4" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B177" s="3" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="C177" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D177" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E177" s="3" t="s">
         <v>52</v>
       </c>
       <c r="F177" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="178" spans="1:6" x14ac:dyDescent="0.3">
@@ -12174,7 +12475,7 @@
         <v>215</v>
       </c>
       <c r="B178" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C178" s="3" t="s">
         <v>37</v>
@@ -12194,7 +12495,7 @@
         <v>215</v>
       </c>
       <c r="B179" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C179" s="3" t="s">
         <v>37</v>
@@ -12203,7 +12504,7 @@
         <v>43</v>
       </c>
       <c r="E179" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F179" s="3" t="s">
         <v>21</v>
@@ -12214,19 +12515,19 @@
         <v>215</v>
       </c>
       <c r="B180" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C180" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D180" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E180" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F180" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.3">
@@ -12234,19 +12535,19 @@
         <v>215</v>
       </c>
       <c r="B181" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C181" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D181" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E181" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F181" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="182" spans="1:6" x14ac:dyDescent="0.3">
@@ -12254,39 +12555,39 @@
         <v>215</v>
       </c>
       <c r="B182" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C182" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D182" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E182" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F182" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="183" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A183" s="4" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="B183" s="3" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="C183" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D183" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E183" s="3" t="s">
         <v>52</v>
       </c>
       <c r="F183" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="184" spans="1:6" x14ac:dyDescent="0.3">
@@ -12294,7 +12595,7 @@
         <v>218</v>
       </c>
       <c r="B184" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C184" s="3" t="s">
         <v>37</v>
@@ -12314,7 +12615,7 @@
         <v>218</v>
       </c>
       <c r="B185" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C185" s="3" t="s">
         <v>37</v>
@@ -12323,7 +12624,7 @@
         <v>43</v>
       </c>
       <c r="E185" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F185" s="3" t="s">
         <v>21</v>
@@ -12334,19 +12635,19 @@
         <v>218</v>
       </c>
       <c r="B186" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C186" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D186" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E186" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F186" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="187" spans="1:6" x14ac:dyDescent="0.3">
@@ -12354,19 +12655,19 @@
         <v>218</v>
       </c>
       <c r="B187" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C187" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D187" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E187" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F187" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="188" spans="1:6" x14ac:dyDescent="0.3">
@@ -12374,27 +12675,27 @@
         <v>218</v>
       </c>
       <c r="B188" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C188" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D188" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E188" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F188" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="189" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A189" s="4" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="B189" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C189" s="3" t="s">
         <v>37</v>
@@ -12414,7 +12715,7 @@
         <v>223</v>
       </c>
       <c r="B190" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C190" s="3" t="s">
         <v>37</v>
@@ -12431,10 +12732,10 @@
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A191" s="4" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B191" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C191" s="3" t="s">
         <v>37</v>
@@ -12454,7 +12755,7 @@
         <v>226</v>
       </c>
       <c r="B192" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C192" s="3" t="s">
         <v>37</v>
@@ -12471,10 +12772,10 @@
     </row>
     <row r="193" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A193" s="4" t="s">
-        <v>226</v>
+        <v>241</v>
       </c>
       <c r="B193" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C193" s="3" t="s">
         <v>37</v>
@@ -12494,7 +12795,7 @@
         <v>241</v>
       </c>
       <c r="B194" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C194" s="3" t="s">
         <v>37</v>
@@ -12511,10 +12812,10 @@
     </row>
     <row r="195" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A195" s="4" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="B195" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C195" s="3" t="s">
         <v>37</v>
@@ -12534,7 +12835,7 @@
         <v>244</v>
       </c>
       <c r="B196" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C196" s="3" t="s">
         <v>37</v>
@@ -12551,10 +12852,10 @@
     </row>
     <row r="197" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A197" s="4" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="B197" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C197" s="3" t="s">
         <v>37</v>
@@ -12574,7 +12875,7 @@
         <v>247</v>
       </c>
       <c r="B198" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C198" s="3" t="s">
         <v>37</v>
@@ -12591,10 +12892,10 @@
     </row>
     <row r="199" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A199" s="4" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="B199" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C199" s="3" t="s">
         <v>37</v>
@@ -12614,7 +12915,7 @@
         <v>251</v>
       </c>
       <c r="B200" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C200" s="3" t="s">
         <v>37</v>
@@ -12631,10 +12932,10 @@
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A201" s="4" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="B201" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C201" s="3" t="s">
         <v>37</v>
@@ -12654,7 +12955,7 @@
         <v>254</v>
       </c>
       <c r="B202" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C202" s="3" t="s">
         <v>37</v>
@@ -12671,10 +12972,10 @@
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A203" s="4" t="s">
-        <v>254</v>
+        <v>272</v>
       </c>
       <c r="B203" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C203" s="3" t="s">
         <v>37</v>
@@ -12694,7 +12995,7 @@
         <v>272</v>
       </c>
       <c r="B204" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C204" s="3" t="s">
         <v>37</v>
@@ -12711,22 +13012,102 @@
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A205" s="4" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="B205" s="3" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="C205" s="3" t="s">
         <v>37</v>
       </c>
       <c r="D205" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E205" s="3" t="s">
         <v>52</v>
       </c>
       <c r="F205" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="206" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A206" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="B206" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C206" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D206" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E206" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F206" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="207" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A207" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="B207" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C207" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D207" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E207" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="F207" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="208" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A208" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="B208" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C208" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D208" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E208" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="F208" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="209" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A209" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B209" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C209" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D209" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E209" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="F209" s="3" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
modified:   recomendador/Tabla_Maestra_ZKTeco.xlsx 	modified:   recomendador/catalogo_zkteco.json 	modified:   recomendador/convertidor.html 	deleted:    recomendador/img/74162.png 	deleted:    recomendador/img/ZKT368012.png 	deleted:    recomendador/img/ZTA065006.png 	new file:   recomendador/img/licencias/BTPFREE.png 	new file:   recomendador/img/licencias/ZLINKFREE.png 	new file:   recomendador/index1.html
</commit_message>
<xml_diff>
--- a/recomendador/Tabla_Maestra_ZKTeco.xlsx
+++ b/recomendador/Tabla_Maestra_ZKTeco.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TVCMTY-57298\Documents\recomendador\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{222444EE-EB6D-484E-B502-BA2B6D796D3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6D907C1-DC66-4D6C-8676-599B23F1DB7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="704" activeTab="4" xr2:uid="{DB513028-4120-4D60-A8C2-889CF1E9B842}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="704" activeTab="5" xr2:uid="{DB513028-4120-4D60-A8C2-889CF1E9B842}"/>
   </bookViews>
   <sheets>
     <sheet name="Equipos" sheetId="1" r:id="rId1"/>
@@ -18,9 +18,12 @@
     <sheet name="Comunicacion" sheetId="3" r:id="rId3"/>
     <sheet name="Software" sheetId="4" r:id="rId4"/>
     <sheet name="Compatibilidad" sheetId="5" r:id="rId5"/>
-    <sheet name="Listas" sheetId="6" r:id="rId6"/>
+    <sheet name="Licencias" sheetId="7" r:id="rId6"/>
+    <sheet name="Licencias_Software" sheetId="8" r:id="rId7"/>
+    <sheet name="Leyenda_Licencias" sheetId="9" r:id="rId8"/>
+    <sheet name="Listas" sheetId="6" r:id="rId9"/>
   </sheets>
-  <calcPr calcId="191029" refMode="R1C1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -42,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3301" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3765" uniqueCount="532">
   <si>
     <t>ID</t>
   </si>
@@ -910,6 +913,755 @@
   </si>
   <si>
     <t>https://tvc.mx/products/88760</t>
+  </si>
+  <si>
+    <t>Clave TVC</t>
+  </si>
+  <si>
+    <t>Licencia</t>
+  </si>
+  <si>
+    <t>Tipo</t>
+  </si>
+  <si>
+    <t>Vigencia</t>
+  </si>
+  <si>
+    <t>Capacidad</t>
+  </si>
+  <si>
+    <t>Checadores</t>
+  </si>
+  <si>
+    <t>Empleados</t>
+  </si>
+  <si>
+    <t>Puertas</t>
+  </si>
+  <si>
+    <t>Requiere</t>
+  </si>
+  <si>
+    <t>Notas</t>
+  </si>
+  <si>
+    <t>BioTime Pro Gratuita (incluida al instalar)</t>
+  </si>
+  <si>
+    <t>Gratuita</t>
+  </si>
+  <si>
+    <t>Vitalicia</t>
+  </si>
+  <si>
+    <t>2 Checadores, 200 Empleados, 1 App y 1 Multiempresa</t>
+  </si>
+  <si>
+    <t>Se activa automáticamente al instalar. Al activar una licencia base, la reemplaza (capacidades no acumulables).</t>
+  </si>
+  <si>
+    <t>ZKT0820003</t>
+  </si>
+  <si>
+    <t>BioTime Pro Starter</t>
+  </si>
+  <si>
+    <t>Base</t>
+  </si>
+  <si>
+    <t>5 Checadores, 500 Empleados, 1 APP y 1 Multicompañía</t>
+  </si>
+  <si>
+    <t>ZKT0820002</t>
+  </si>
+  <si>
+    <t>BioTime Pro Lite</t>
+  </si>
+  <si>
+    <t>10 Checadores, 1000 Empleados, 1 APP y 1 Multicompañía</t>
+  </si>
+  <si>
+    <t>ZKT0820004</t>
+  </si>
+  <si>
+    <t>BioTime Pro Standard</t>
+  </si>
+  <si>
+    <t>20 Checadores, 2000 Empleados, 1 APP y 2 Multicompañías</t>
+  </si>
+  <si>
+    <t>ZKT0820005</t>
+  </si>
+  <si>
+    <t>BioTime Pro Premium</t>
+  </si>
+  <si>
+    <t>50 Checadores, 6000 Empleados, 1 APP y 5 Multicompañías</t>
+  </si>
+  <si>
+    <t>ZKT0820006</t>
+  </si>
+  <si>
+    <t>BioTime Pro Prime</t>
+  </si>
+  <si>
+    <t>75 Checadores, 8000 Empleados, 1 APP y 7 Multicompañías</t>
+  </si>
+  <si>
+    <t>ZKT0820007</t>
+  </si>
+  <si>
+    <t>BioTime Pro Enterprise</t>
+  </si>
+  <si>
+    <t>100 Checadores, 12000 Empleados, 1 APP y 10 Multicompañías</t>
+  </si>
+  <si>
+    <t>ZKT0820008</t>
+  </si>
+  <si>
+    <t>BioTime Pro Business</t>
+  </si>
+  <si>
+    <t>150 Checadores, 15000 Empleados, 1 APP y 15 Multicompañías</t>
+  </si>
+  <si>
+    <t>ZKT0820009</t>
+  </si>
+  <si>
+    <t>BioTime Pro Professional</t>
+  </si>
+  <si>
+    <t>200 Checadores, 20000 Empleados, 1 APP y 20 Multicompañías</t>
+  </si>
+  <si>
+    <t>ZKT0820010</t>
+  </si>
+  <si>
+    <t>BioTime Pro Big Project</t>
+  </si>
+  <si>
+    <t>300 Checadores, 30000 Empleados, 1 APP y 30 Multicompañías</t>
+  </si>
+  <si>
+    <t>ZKT0820011</t>
+  </si>
+  <si>
+    <t>BioTime Pro Great Project</t>
+  </si>
+  <si>
+    <t>500 Checadores, 50000 Empleados, 1 APP y 50 Multicompañías</t>
+  </si>
+  <si>
+    <t>ZKT0820012</t>
+  </si>
+  <si>
+    <t>BioTime Pro Ultimate</t>
+  </si>
+  <si>
+    <t>800 Checadores, 80000 Empleados, 1 APP y 50 Multicompañías</t>
+  </si>
+  <si>
+    <t>ZKT0820015</t>
+  </si>
+  <si>
+    <t>BioTime Pro App Basic</t>
+  </si>
+  <si>
+    <t>App</t>
+  </si>
+  <si>
+    <t>20 APPs</t>
+  </si>
+  <si>
+    <t>Licencia base que soporte la cantidad de APPs móviles</t>
+  </si>
+  <si>
+    <t>ZKT0820016</t>
+  </si>
+  <si>
+    <t>BioTime Pro App Lite</t>
+  </si>
+  <si>
+    <t>50 APPs</t>
+  </si>
+  <si>
+    <t>ZKT0820017</t>
+  </si>
+  <si>
+    <t>BioTime Pro App Standard</t>
+  </si>
+  <si>
+    <t>100 APPs</t>
+  </si>
+  <si>
+    <t>ZKT0820018</t>
+  </si>
+  <si>
+    <t>BioTime Pro App Professional</t>
+  </si>
+  <si>
+    <t>200 APPs</t>
+  </si>
+  <si>
+    <t>ZKT0820019</t>
+  </si>
+  <si>
+    <t>BioTime Pro App Premium</t>
+  </si>
+  <si>
+    <t>300 APPs</t>
+  </si>
+  <si>
+    <t>ZKT0820020</t>
+  </si>
+  <si>
+    <t>BioTime Pro App Enterprise</t>
+  </si>
+  <si>
+    <t>500 APPs</t>
+  </si>
+  <si>
+    <t>ZKT0820021</t>
+  </si>
+  <si>
+    <t>BioTime Pro App Business</t>
+  </si>
+  <si>
+    <t>800 APPs</t>
+  </si>
+  <si>
+    <t>ZKT0820014</t>
+  </si>
+  <si>
+    <t>BioTime Pro Additional User</t>
+  </si>
+  <si>
+    <t>Aumento</t>
+  </si>
+  <si>
+    <t>1 Empleado adicional</t>
+  </si>
+  <si>
+    <t>Licencia base</t>
+  </si>
+  <si>
+    <t>ZKT0820013</t>
+  </si>
+  <si>
+    <t>BioTime Pro Additional Devices</t>
+  </si>
+  <si>
+    <t>5 Checadores adicionales</t>
+  </si>
+  <si>
+    <t>ZKT0820026</t>
+  </si>
+  <si>
+    <t>BioTime Pro Additional Company</t>
+  </si>
+  <si>
+    <t>1 Compañía adicional</t>
+  </si>
+  <si>
+    <t>ZKT0820146</t>
+  </si>
+  <si>
+    <t>BioTime Cloud 2.0 Lite</t>
+  </si>
+  <si>
+    <t>Suscripción</t>
+  </si>
+  <si>
+    <t>Anual</t>
+  </si>
+  <si>
+    <t>3 Checadores, 25 Empleados, 10 APPs y 37500 Eventos</t>
+  </si>
+  <si>
+    <t>ZKT0820147</t>
+  </si>
+  <si>
+    <t>BioTime Cloud 2.0 Standard</t>
+  </si>
+  <si>
+    <t>6 Checadores, 50 Empleados, 25 APPs y 75000 Eventos</t>
+  </si>
+  <si>
+    <t>ZKT0820148</t>
+  </si>
+  <si>
+    <t>BioTime Cloud 2.0 Professional</t>
+  </si>
+  <si>
+    <t>15 Checadores, 100 Empleados, 75 APPs y 150000 Eventos</t>
+  </si>
+  <si>
+    <t>ZKT0820149</t>
+  </si>
+  <si>
+    <t>BioTime Cloud 2.0 Enterprise</t>
+  </si>
+  <si>
+    <t>40 Checadores, 300 Empleados, 300 APPs y 450000 Eventos</t>
+  </si>
+  <si>
+    <t>ZKT0820150</t>
+  </si>
+  <si>
+    <t>BioTime Cloud 2.0 Premium</t>
+  </si>
+  <si>
+    <t>60 Checadores, 500 Empleados, 500 APPs y 750000 Eventos</t>
+  </si>
+  <si>
+    <t>ZKT0740100</t>
+  </si>
+  <si>
+    <t>ZKCVA-FREE</t>
+  </si>
+  <si>
+    <t>Acceso/Asistencia</t>
+  </si>
+  <si>
+    <t>2000 Empleados, 15 Puertas de Acceso, 6 Checadores, 64 Canales de Video, 1 APP de Administrador y 5 APPs de Empleados</t>
+  </si>
+  <si>
+    <t>Sin costo al adquirir equipos compatibles (validar elegibilidad con el asesor). Existen licencias con costo hasta 25 puertas, 25 puntos de asistencia o 4,000 usuarios (consultar clave y costo con el asesor).</t>
+  </si>
+  <si>
+    <t>ZKT0740042</t>
+  </si>
+  <si>
+    <t>ZKBioCV-AC-P5</t>
+  </si>
+  <si>
+    <t>5 Puertas de Acceso</t>
+  </si>
+  <si>
+    <t>Incluye 30,000 empleados, 2,000 departamentos, 2,000 áreas, APIs activas, 1 App de administrador, 50 Apps de empleados y 64 canales de video (salvo indicación).</t>
+  </si>
+  <si>
+    <t>ZKT0740043</t>
+  </si>
+  <si>
+    <t>ZKBioCV-AC-P10</t>
+  </si>
+  <si>
+    <t>10 Puertas de Acceso</t>
+  </si>
+  <si>
+    <t>ZKT0740044</t>
+  </si>
+  <si>
+    <t>ZKBioCV-AC-P25</t>
+  </si>
+  <si>
+    <t>25 Puertas de Acceso</t>
+  </si>
+  <si>
+    <t>ZKT0740045</t>
+  </si>
+  <si>
+    <t>ZKBioCV-AC-P50</t>
+  </si>
+  <si>
+    <t>50 Puertas de Acceso</t>
+  </si>
+  <si>
+    <t>ZKT0740046</t>
+  </si>
+  <si>
+    <t>ZKBioCV-AC-P75</t>
+  </si>
+  <si>
+    <t>75 Puertas de Acceso</t>
+  </si>
+  <si>
+    <t>ZKT0740047</t>
+  </si>
+  <si>
+    <t>ZKBioCV-AC-P100</t>
+  </si>
+  <si>
+    <t>100 Puertas de Acceso</t>
+  </si>
+  <si>
+    <t>ZKT0740119</t>
+  </si>
+  <si>
+    <t>ZKBioCV-AC-P150</t>
+  </si>
+  <si>
+    <t>150 Puertas de Acceso</t>
+  </si>
+  <si>
+    <t>ZKT0740118</t>
+  </si>
+  <si>
+    <t>ZKBioCV-AC-P200</t>
+  </si>
+  <si>
+    <t>200 Puertas de Acceso</t>
+  </si>
+  <si>
+    <t>ZKT0740115</t>
+  </si>
+  <si>
+    <t>ZKBioCV-AC-P250</t>
+  </si>
+  <si>
+    <t>250 Puertas de Acceso</t>
+  </si>
+  <si>
+    <t>ZKT0740049</t>
+  </si>
+  <si>
+    <t>ZKBioCV-AC-ADDON-P5</t>
+  </si>
+  <si>
+    <t>5 Puertas de Acceso Adicionales</t>
+  </si>
+  <si>
+    <t>Licencia base de 25 puertas o superior</t>
+  </si>
+  <si>
+    <t>ZKT0820112</t>
+  </si>
+  <si>
+    <t>ZKBioCV-TA-P5</t>
+  </si>
+  <si>
+    <t>5 Checadores</t>
+  </si>
+  <si>
+    <t>ZKT0820113</t>
+  </si>
+  <si>
+    <t>ZKBioCV-TA-P10</t>
+  </si>
+  <si>
+    <t>10 Checadores</t>
+  </si>
+  <si>
+    <t>ZKT0820114</t>
+  </si>
+  <si>
+    <t>ZKBioCV-TA-P25</t>
+  </si>
+  <si>
+    <t>25 Checadores</t>
+  </si>
+  <si>
+    <t>ZKT0820115</t>
+  </si>
+  <si>
+    <t>ZKBioCV-TA-P50</t>
+  </si>
+  <si>
+    <t>50 Checadores</t>
+  </si>
+  <si>
+    <t>ZKT0820116</t>
+  </si>
+  <si>
+    <t>ZKBioCV-TA-P75</t>
+  </si>
+  <si>
+    <t>75 Checadores</t>
+  </si>
+  <si>
+    <t>ZKT0820117</t>
+  </si>
+  <si>
+    <t>ZKBioCV-TA-P100</t>
+  </si>
+  <si>
+    <t>100 Checadores</t>
+  </si>
+  <si>
+    <t>ZKT0820118</t>
+  </si>
+  <si>
+    <t>ZKBioCV-TA-ADDON-P5</t>
+  </si>
+  <si>
+    <t>5 Checadores Adicionales</t>
+  </si>
+  <si>
+    <t>Licencia base de 25 checadores o superior</t>
+  </si>
+  <si>
+    <t>ZKBio Zlink (gratuito)</t>
+  </si>
+  <si>
+    <t>Software gratuito para equipos con protocolo BEST (sin clave TVC)</t>
+  </si>
+  <si>
+    <t>Compatible con equipos en protocolo BEST.</t>
+  </si>
+  <si>
+    <t>Descripción</t>
+  </si>
+  <si>
+    <t>Despliegue</t>
+  </si>
+  <si>
+    <t>Control de asistencia mediante protocolo PUSH con licenciamiento vitalicio.</t>
+  </si>
+  <si>
+    <t>Local</t>
+  </si>
+  <si>
+    <t>Incluye versión gratuita automática (2 checadores, 200 empleados, 1 App, 1 multiempresa); al activar una licencia base la reemplaza y las capacidades no son acumulables.
+Las licencias de aumento requieren licencia base y un proceso de unificación (copia de la licencia base activa); durante la unificación la licencia puede quedar temporalmente deshabilitada.
+No es posible unificar dos o más licencias base entre sí; para crecer se usan licencias de aumento.
+Migración de servidor o falla de hardware: reset de licencia gratuito (si no se detecta uso indebido).
+Procesar licencia, reset o unificación toma de 3 a 5 días hábiles. No se aceptan devoluciones.</t>
+  </si>
+  <si>
+    <t>Plataforma de control de asistencia en la nube (AWS) mediante protocolo PUSH, por suscripción anual.</t>
+  </si>
+  <si>
+    <t>Nube</t>
+  </si>
+  <si>
+    <t>No requiere instalación: se accede desde un navegador web. No hay proceso de reset de licencia.
+No se pueden combinar ni unificar suscripciones; tampoco ampliar terminales, empleados o apps de una suscripción (hay que adquirir una de mayor capacidad, que reemplaza la actual).
+La capacidad de eventos sí puede ampliarse de forma permanente con una actualización adicional.
+Activación de 3 a 5 días hábiles. No se aceptan devoluciones.</t>
+  </si>
+  <si>
+    <t>Software ligero WEB para pequeñas y medianas empresas, con licencia vitalicia base.</t>
+  </si>
+  <si>
+    <t>Local (Web)</t>
+  </si>
+  <si>
+    <t>La licencia gratuita se obtiene al adquirir equipos compatibles; validar elegibilidad con el asesor.
+Con costo existen licencias para ampliar hasta 25 puertas, 25 puntos de asistencia o 4,000 usuarios (consultar clave TVC y costo).
+Si el proyecto requiere más capacidad, evaluar ZKBio CVSecurity.
+Reset gratuito en migración o falla de hardware (si no hay uso indebido). 3 a 5 días hábiles. No se aceptan devoluciones.</t>
+  </si>
+  <si>
+    <t>Software modular para soluciones escalables y robustas, con licencias vitalicias cotizables por módulo.</t>
+  </si>
+  <si>
+    <t>Salvo indicación, las licencias base incluyen 30,000 empleados, 2,000 departamentos, 2,000 áreas, APIs activas, 1 App de administrador, 50 Apps de empleados y 64 canales de video.
+Aumentos de Acceso o Asistencia requieren unificación con la licencia base (copia de la licencia activa); la licencia puede quedar temporalmente deshabilitada durante el proceso.
+Se pueden unificar licencias de distintos módulos en una misma instalación, pero no dos o más bases del mismo módulo (Acceso, Asistencia, Visitas, Patrullaje y Hotel).
+Patrullaje requiere licencia activa en el Módulo de Acceso.
+Reset gratuito (si no hay uso indebido). 3 a 5 días hábiles. No se aceptan devoluciones.</t>
+  </si>
+  <si>
+    <t>Software gratuito para equipos con protocolo BEST.</t>
+  </si>
+  <si>
+    <t>Gratuito, sin clave TVC. Para equipos que trabajan con protocolo BEST.</t>
+  </si>
+  <si>
+    <t>Hoja</t>
+  </si>
+  <si>
+    <t>Qué contiene</t>
+  </si>
+  <si>
+    <t>Licencias</t>
+  </si>
+  <si>
+    <t>Una fila por licencia (clave TVC). Copia esta hoja a tu Tabla_Maestra_ZKTeco.xlsx con el mismo nombre y encabezados.</t>
+  </si>
+  <si>
+    <t>Licencias_Software</t>
+  </si>
+  <si>
+    <t>Una fila por software: descripción, despliegue y "puntos importantes" (una nota por renglón dentro de la celda).</t>
+  </si>
+  <si>
+    <t>Columna (Licencias)</t>
+  </si>
+  <si>
+    <t>Cómo llenarla</t>
+  </si>
+  <si>
+    <t>Clave del producto. Vacía si es gratuita o sin clave (ej. ZKBio Zlink, versión gratuita de BioTime Pro).</t>
+  </si>
+  <si>
+    <t>Nombre visible de la licencia.</t>
+  </si>
+  <si>
+    <t>Debe escribirse igual (o casi igual) que en la hoja "Software" de la tabla maestra: así se cruza con los equipos compatibles (ej. "BioTime Pro", "ZKBio CVSecurity").</t>
+  </si>
+  <si>
+    <t>Acceso, Asistencia, Visitas, etc. Si aplica a varios: "Acceso/Asistencia". Solo Acceso y Asistencia se cruzan por módulo con la hoja Compatibilidad; los demás módulos se cruzan por software.</t>
+  </si>
+  <si>
+    <t>Base, Aumento, App, Suscripción, Gratuita o Bajo proyecto.</t>
+  </si>
+  <si>
+    <t>Vitalicia, Anual, 36 meses, 1 año, Gratuita (o vacío si no se indica).</t>
+  </si>
+  <si>
+    <t>Texto libre con la capacidad tal como se presenta al cliente.</t>
+  </si>
+  <si>
+    <t>Checadores / Empleados / Puertas</t>
+  </si>
+  <si>
+    <t>Números (opcionales) usados por los filtros de capacidad mínima. Déjalos vacíos si no aplican.</t>
+  </si>
+  <si>
+    <t>Texto libre con requisitos (ej. "Licencia base de 25 puertas o superior").</t>
+  </si>
+  <si>
+    <t>Texto libre adicional.</t>
+  </si>
+  <si>
+    <t>Ilimitadas</t>
+  </si>
+  <si>
+    <t>APPs</t>
+  </si>
+  <si>
+    <t>Imagen</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/49130</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/68070</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/31258</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/31298</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/31262</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/31318</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/31306</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/70895</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/70890</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/70900</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/70905</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/70910</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/31302</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/31322</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/33486</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/31330</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/31286</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/31282</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/31270</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/31326</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/31310</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/31274</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/31254</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/31266</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/31278</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/31290</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/31294</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/31314</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/49135</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/49140</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/49175</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/49150</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/49145</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/80492</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/80487</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/79550</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/49160</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/49180</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/49190</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/49205</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/49200</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/49210</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/49195</t>
+  </si>
+  <si>
+    <t>https://tvc.mx/products/49185</t>
+  </si>
+  <si>
+    <t>img/licencias/BTPFREE.png</t>
+  </si>
+  <si>
+    <t>img/licencias/ZLINKFREE.png</t>
   </si>
 </sst>
 </file>
@@ -959,7 +1711,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -988,6 +1740,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4655,7 +5412,7 @@
         <v>23</v>
       </c>
       <c r="P44" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="Q44" s="5" t="s">
         <v>20</v>
@@ -13117,6 +13874,1930 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4323FEF8-9A72-43CC-8BE6-9B44175C2B39}">
+  <dimension ref="A1:Q47"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="48.33203125" customWidth="1"/>
+    <col min="5" max="5" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="108" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="48.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="176.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>287</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>485</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="G1" s="11" t="s">
+        <v>289</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>290</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>291</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>292</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>293</v>
+      </c>
+      <c r="L1" s="11" t="s">
+        <v>294</v>
+      </c>
+      <c r="M1" s="11" t="s">
+        <v>484</v>
+      </c>
+      <c r="N1" s="11" t="s">
+        <v>295</v>
+      </c>
+      <c r="Q1" s="11" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="B2" t="s">
+        <v>297</v>
+      </c>
+      <c r="C2" t="s">
+        <v>530</v>
+      </c>
+      <c r="E2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F2" t="s">
+        <v>43</v>
+      </c>
+      <c r="G2" t="s">
+        <v>298</v>
+      </c>
+      <c r="H2" t="s">
+        <v>299</v>
+      </c>
+      <c r="I2" t="s">
+        <v>300</v>
+      </c>
+      <c r="J2">
+        <v>2</v>
+      </c>
+      <c r="K2">
+        <v>200</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>302</v>
+      </c>
+      <c r="B3" t="s">
+        <v>303</v>
+      </c>
+      <c r="D3" t="s">
+        <v>488</v>
+      </c>
+      <c r="E3" t="s">
+        <v>51</v>
+      </c>
+      <c r="F3" t="s">
+        <v>43</v>
+      </c>
+      <c r="G3" t="s">
+        <v>304</v>
+      </c>
+      <c r="H3" t="s">
+        <v>299</v>
+      </c>
+      <c r="I3" t="s">
+        <v>305</v>
+      </c>
+      <c r="J3">
+        <v>5</v>
+      </c>
+      <c r="K3">
+        <v>500</v>
+      </c>
+      <c r="M3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>306</v>
+      </c>
+      <c r="B4" t="s">
+        <v>307</v>
+      </c>
+      <c r="D4" t="s">
+        <v>508</v>
+      </c>
+      <c r="E4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F4" t="s">
+        <v>43</v>
+      </c>
+      <c r="G4" t="s">
+        <v>304</v>
+      </c>
+      <c r="H4" t="s">
+        <v>299</v>
+      </c>
+      <c r="I4" t="s">
+        <v>308</v>
+      </c>
+      <c r="J4">
+        <v>10</v>
+      </c>
+      <c r="K4">
+        <v>1000</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>309</v>
+      </c>
+      <c r="B5" t="s">
+        <v>310</v>
+      </c>
+      <c r="D5" t="s">
+        <v>490</v>
+      </c>
+      <c r="E5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F5" t="s">
+        <v>43</v>
+      </c>
+      <c r="G5" t="s">
+        <v>304</v>
+      </c>
+      <c r="H5" t="s">
+        <v>299</v>
+      </c>
+      <c r="I5" t="s">
+        <v>311</v>
+      </c>
+      <c r="J5">
+        <v>20</v>
+      </c>
+      <c r="K5">
+        <v>2000</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>312</v>
+      </c>
+      <c r="B6" t="s">
+        <v>313</v>
+      </c>
+      <c r="D6" t="s">
+        <v>509</v>
+      </c>
+      <c r="E6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F6" t="s">
+        <v>43</v>
+      </c>
+      <c r="G6" t="s">
+        <v>304</v>
+      </c>
+      <c r="H6" t="s">
+        <v>299</v>
+      </c>
+      <c r="I6" t="s">
+        <v>314</v>
+      </c>
+      <c r="J6">
+        <v>50</v>
+      </c>
+      <c r="K6">
+        <v>6000</v>
+      </c>
+      <c r="M6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>315</v>
+      </c>
+      <c r="B7" t="s">
+        <v>316</v>
+      </c>
+      <c r="D7" t="s">
+        <v>504</v>
+      </c>
+      <c r="E7" t="s">
+        <v>51</v>
+      </c>
+      <c r="F7" t="s">
+        <v>43</v>
+      </c>
+      <c r="G7" t="s">
+        <v>304</v>
+      </c>
+      <c r="H7" t="s">
+        <v>299</v>
+      </c>
+      <c r="I7" t="s">
+        <v>317</v>
+      </c>
+      <c r="J7">
+        <v>75</v>
+      </c>
+      <c r="K7">
+        <v>8000</v>
+      </c>
+      <c r="M7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>318</v>
+      </c>
+      <c r="B8" t="s">
+        <v>319</v>
+      </c>
+      <c r="D8" t="s">
+        <v>507</v>
+      </c>
+      <c r="E8" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" t="s">
+        <v>43</v>
+      </c>
+      <c r="G8" t="s">
+        <v>304</v>
+      </c>
+      <c r="H8" t="s">
+        <v>299</v>
+      </c>
+      <c r="I8" t="s">
+        <v>320</v>
+      </c>
+      <c r="J8">
+        <v>100</v>
+      </c>
+      <c r="K8">
+        <v>12000</v>
+      </c>
+      <c r="M8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>321</v>
+      </c>
+      <c r="B9" t="s">
+        <v>322</v>
+      </c>
+      <c r="D9" t="s">
+        <v>510</v>
+      </c>
+      <c r="E9" t="s">
+        <v>51</v>
+      </c>
+      <c r="F9" t="s">
+        <v>43</v>
+      </c>
+      <c r="G9" t="s">
+        <v>304</v>
+      </c>
+      <c r="H9" t="s">
+        <v>299</v>
+      </c>
+      <c r="I9" t="s">
+        <v>323</v>
+      </c>
+      <c r="J9">
+        <v>150</v>
+      </c>
+      <c r="K9">
+        <v>15000</v>
+      </c>
+      <c r="M9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>324</v>
+      </c>
+      <c r="B10" t="s">
+        <v>325</v>
+      </c>
+      <c r="D10" t="s">
+        <v>503</v>
+      </c>
+      <c r="E10" t="s">
+        <v>51</v>
+      </c>
+      <c r="F10" t="s">
+        <v>43</v>
+      </c>
+      <c r="G10" t="s">
+        <v>304</v>
+      </c>
+      <c r="H10" t="s">
+        <v>299</v>
+      </c>
+      <c r="I10" t="s">
+        <v>326</v>
+      </c>
+      <c r="J10">
+        <v>200</v>
+      </c>
+      <c r="K10">
+        <v>20000</v>
+      </c>
+      <c r="M10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>327</v>
+      </c>
+      <c r="B11" t="s">
+        <v>328</v>
+      </c>
+      <c r="D11" t="s">
+        <v>502</v>
+      </c>
+      <c r="E11" t="s">
+        <v>51</v>
+      </c>
+      <c r="F11" t="s">
+        <v>43</v>
+      </c>
+      <c r="G11" t="s">
+        <v>304</v>
+      </c>
+      <c r="H11" t="s">
+        <v>299</v>
+      </c>
+      <c r="I11" t="s">
+        <v>329</v>
+      </c>
+      <c r="J11">
+        <v>300</v>
+      </c>
+      <c r="K11">
+        <v>30000</v>
+      </c>
+      <c r="M11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>330</v>
+      </c>
+      <c r="B12" t="s">
+        <v>331</v>
+      </c>
+      <c r="D12" t="s">
+        <v>511</v>
+      </c>
+      <c r="E12" t="s">
+        <v>51</v>
+      </c>
+      <c r="F12" t="s">
+        <v>43</v>
+      </c>
+      <c r="G12" t="s">
+        <v>304</v>
+      </c>
+      <c r="H12" t="s">
+        <v>299</v>
+      </c>
+      <c r="I12" t="s">
+        <v>332</v>
+      </c>
+      <c r="J12">
+        <v>500</v>
+      </c>
+      <c r="K12">
+        <v>50000</v>
+      </c>
+      <c r="M12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>333</v>
+      </c>
+      <c r="B13" t="s">
+        <v>334</v>
+      </c>
+      <c r="D13" t="s">
+        <v>512</v>
+      </c>
+      <c r="E13" t="s">
+        <v>51</v>
+      </c>
+      <c r="F13" t="s">
+        <v>43</v>
+      </c>
+      <c r="G13" t="s">
+        <v>304</v>
+      </c>
+      <c r="H13" t="s">
+        <v>299</v>
+      </c>
+      <c r="I13" t="s">
+        <v>335</v>
+      </c>
+      <c r="J13">
+        <v>800</v>
+      </c>
+      <c r="K13">
+        <v>80000</v>
+      </c>
+      <c r="M13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>336</v>
+      </c>
+      <c r="B14" t="s">
+        <v>337</v>
+      </c>
+      <c r="D14" t="s">
+        <v>492</v>
+      </c>
+      <c r="E14" t="s">
+        <v>51</v>
+      </c>
+      <c r="F14" t="s">
+        <v>43</v>
+      </c>
+      <c r="G14" t="s">
+        <v>338</v>
+      </c>
+      <c r="H14" t="s">
+        <v>299</v>
+      </c>
+      <c r="I14" t="s">
+        <v>339</v>
+      </c>
+      <c r="M14">
+        <v>20</v>
+      </c>
+      <c r="N14" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>341</v>
+      </c>
+      <c r="B15" t="s">
+        <v>342</v>
+      </c>
+      <c r="D15" t="s">
+        <v>506</v>
+      </c>
+      <c r="E15" t="s">
+        <v>51</v>
+      </c>
+      <c r="F15" t="s">
+        <v>43</v>
+      </c>
+      <c r="G15" t="s">
+        <v>338</v>
+      </c>
+      <c r="H15" t="s">
+        <v>299</v>
+      </c>
+      <c r="I15" t="s">
+        <v>343</v>
+      </c>
+      <c r="M15">
+        <v>50</v>
+      </c>
+      <c r="N15" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>344</v>
+      </c>
+      <c r="B16" t="s">
+        <v>345</v>
+      </c>
+      <c r="D16" t="s">
+        <v>513</v>
+      </c>
+      <c r="E16" t="s">
+        <v>51</v>
+      </c>
+      <c r="F16" t="s">
+        <v>43</v>
+      </c>
+      <c r="G16" t="s">
+        <v>338</v>
+      </c>
+      <c r="H16" t="s">
+        <v>299</v>
+      </c>
+      <c r="I16" t="s">
+        <v>346</v>
+      </c>
+      <c r="M16">
+        <v>100</v>
+      </c>
+      <c r="N16" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>347</v>
+      </c>
+      <c r="B17" t="s">
+        <v>348</v>
+      </c>
+      <c r="D17" t="s">
+        <v>491</v>
+      </c>
+      <c r="E17" t="s">
+        <v>51</v>
+      </c>
+      <c r="F17" t="s">
+        <v>43</v>
+      </c>
+      <c r="G17" t="s">
+        <v>338</v>
+      </c>
+      <c r="H17" t="s">
+        <v>299</v>
+      </c>
+      <c r="I17" t="s">
+        <v>349</v>
+      </c>
+      <c r="M17">
+        <v>200</v>
+      </c>
+      <c r="N17" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>350</v>
+      </c>
+      <c r="B18" t="s">
+        <v>351</v>
+      </c>
+      <c r="D18" t="s">
+        <v>499</v>
+      </c>
+      <c r="E18" t="s">
+        <v>51</v>
+      </c>
+      <c r="F18" t="s">
+        <v>43</v>
+      </c>
+      <c r="G18" t="s">
+        <v>338</v>
+      </c>
+      <c r="H18" t="s">
+        <v>299</v>
+      </c>
+      <c r="I18" t="s">
+        <v>352</v>
+      </c>
+      <c r="M18">
+        <v>300</v>
+      </c>
+      <c r="N18" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>353</v>
+      </c>
+      <c r="B19" t="s">
+        <v>354</v>
+      </c>
+      <c r="D19" t="s">
+        <v>505</v>
+      </c>
+      <c r="E19" t="s">
+        <v>51</v>
+      </c>
+      <c r="F19" t="s">
+        <v>43</v>
+      </c>
+      <c r="G19" t="s">
+        <v>338</v>
+      </c>
+      <c r="H19" t="s">
+        <v>299</v>
+      </c>
+      <c r="I19" t="s">
+        <v>355</v>
+      </c>
+      <c r="M19">
+        <v>500</v>
+      </c>
+      <c r="N19" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>356</v>
+      </c>
+      <c r="B20" t="s">
+        <v>357</v>
+      </c>
+      <c r="D20" t="s">
+        <v>501</v>
+      </c>
+      <c r="E20" t="s">
+        <v>51</v>
+      </c>
+      <c r="F20" t="s">
+        <v>43</v>
+      </c>
+      <c r="G20" t="s">
+        <v>338</v>
+      </c>
+      <c r="H20" t="s">
+        <v>299</v>
+      </c>
+      <c r="I20" t="s">
+        <v>358</v>
+      </c>
+      <c r="M20">
+        <v>800</v>
+      </c>
+      <c r="N20" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>359</v>
+      </c>
+      <c r="B21" t="s">
+        <v>360</v>
+      </c>
+      <c r="D21" t="s">
+        <v>498</v>
+      </c>
+      <c r="E21" t="s">
+        <v>51</v>
+      </c>
+      <c r="F21" t="s">
+        <v>43</v>
+      </c>
+      <c r="G21" t="s">
+        <v>361</v>
+      </c>
+      <c r="H21" t="s">
+        <v>299</v>
+      </c>
+      <c r="I21" t="s">
+        <v>362</v>
+      </c>
+      <c r="K21">
+        <v>1</v>
+      </c>
+      <c r="N21" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>364</v>
+      </c>
+      <c r="B22" t="s">
+        <v>365</v>
+      </c>
+      <c r="D22" t="s">
+        <v>489</v>
+      </c>
+      <c r="E22" t="s">
+        <v>51</v>
+      </c>
+      <c r="F22" t="s">
+        <v>43</v>
+      </c>
+      <c r="G22" t="s">
+        <v>361</v>
+      </c>
+      <c r="H22" t="s">
+        <v>299</v>
+      </c>
+      <c r="I22" t="s">
+        <v>366</v>
+      </c>
+      <c r="J22">
+        <v>5</v>
+      </c>
+      <c r="N22" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>367</v>
+      </c>
+      <c r="B23" t="s">
+        <v>368</v>
+      </c>
+      <c r="D23" t="s">
+        <v>500</v>
+      </c>
+      <c r="E23" t="s">
+        <v>51</v>
+      </c>
+      <c r="F23" t="s">
+        <v>43</v>
+      </c>
+      <c r="G23" t="s">
+        <v>361</v>
+      </c>
+      <c r="H23" t="s">
+        <v>299</v>
+      </c>
+      <c r="I23" t="s">
+        <v>369</v>
+      </c>
+      <c r="N23" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>370</v>
+      </c>
+      <c r="B24" t="s">
+        <v>371</v>
+      </c>
+      <c r="D24" t="s">
+        <v>494</v>
+      </c>
+      <c r="E24" t="s">
+        <v>54</v>
+      </c>
+      <c r="F24" t="s">
+        <v>43</v>
+      </c>
+      <c r="G24" t="s">
+        <v>372</v>
+      </c>
+      <c r="H24" t="s">
+        <v>373</v>
+      </c>
+      <c r="I24" t="s">
+        <v>374</v>
+      </c>
+      <c r="J24">
+        <v>3</v>
+      </c>
+      <c r="K24">
+        <v>25</v>
+      </c>
+      <c r="M24">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>375</v>
+      </c>
+      <c r="B25" t="s">
+        <v>376</v>
+      </c>
+      <c r="D25" t="s">
+        <v>493</v>
+      </c>
+      <c r="E25" t="s">
+        <v>54</v>
+      </c>
+      <c r="F25" t="s">
+        <v>43</v>
+      </c>
+      <c r="G25" t="s">
+        <v>372</v>
+      </c>
+      <c r="H25" t="s">
+        <v>373</v>
+      </c>
+      <c r="I25" t="s">
+        <v>377</v>
+      </c>
+      <c r="J25">
+        <v>6</v>
+      </c>
+      <c r="K25">
+        <v>50</v>
+      </c>
+      <c r="M25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>378</v>
+      </c>
+      <c r="B26" t="s">
+        <v>379</v>
+      </c>
+      <c r="D26" t="s">
+        <v>495</v>
+      </c>
+      <c r="E26" t="s">
+        <v>54</v>
+      </c>
+      <c r="F26" t="s">
+        <v>43</v>
+      </c>
+      <c r="G26" t="s">
+        <v>372</v>
+      </c>
+      <c r="H26" t="s">
+        <v>373</v>
+      </c>
+      <c r="I26" t="s">
+        <v>380</v>
+      </c>
+      <c r="J26">
+        <v>15</v>
+      </c>
+      <c r="K26">
+        <v>100</v>
+      </c>
+      <c r="M26">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>381</v>
+      </c>
+      <c r="B27" t="s">
+        <v>382</v>
+      </c>
+      <c r="D27" t="s">
+        <v>496</v>
+      </c>
+      <c r="E27" t="s">
+        <v>54</v>
+      </c>
+      <c r="F27" t="s">
+        <v>43</v>
+      </c>
+      <c r="G27" t="s">
+        <v>372</v>
+      </c>
+      <c r="H27" t="s">
+        <v>373</v>
+      </c>
+      <c r="I27" t="s">
+        <v>383</v>
+      </c>
+      <c r="J27">
+        <v>40</v>
+      </c>
+      <c r="K27">
+        <v>300</v>
+      </c>
+      <c r="M27">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>384</v>
+      </c>
+      <c r="B28" t="s">
+        <v>385</v>
+      </c>
+      <c r="D28" t="s">
+        <v>497</v>
+      </c>
+      <c r="E28" t="s">
+        <v>54</v>
+      </c>
+      <c r="F28" t="s">
+        <v>43</v>
+      </c>
+      <c r="G28" t="s">
+        <v>372</v>
+      </c>
+      <c r="H28" t="s">
+        <v>373</v>
+      </c>
+      <c r="I28" t="s">
+        <v>386</v>
+      </c>
+      <c r="J28">
+        <v>60</v>
+      </c>
+      <c r="K28">
+        <v>500</v>
+      </c>
+      <c r="M28">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>387</v>
+      </c>
+      <c r="B29" t="s">
+        <v>388</v>
+      </c>
+      <c r="D29" t="s">
+        <v>487</v>
+      </c>
+      <c r="E29" t="s">
+        <v>56</v>
+      </c>
+      <c r="F29" t="s">
+        <v>389</v>
+      </c>
+      <c r="G29" t="s">
+        <v>298</v>
+      </c>
+      <c r="H29" t="s">
+        <v>299</v>
+      </c>
+      <c r="I29" t="s">
+        <v>390</v>
+      </c>
+      <c r="J29">
+        <v>6</v>
+      </c>
+      <c r="K29">
+        <v>2000</v>
+      </c>
+      <c r="L29">
+        <v>15</v>
+      </c>
+      <c r="M29">
+        <v>5</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>392</v>
+      </c>
+      <c r="B30" t="s">
+        <v>393</v>
+      </c>
+      <c r="D30" t="s">
+        <v>486</v>
+      </c>
+      <c r="E30" t="s">
+        <v>60</v>
+      </c>
+      <c r="F30" t="s">
+        <v>44</v>
+      </c>
+      <c r="G30" t="s">
+        <v>304</v>
+      </c>
+      <c r="H30" t="s">
+        <v>299</v>
+      </c>
+      <c r="I30" t="s">
+        <v>394</v>
+      </c>
+      <c r="K30">
+        <v>30000</v>
+      </c>
+      <c r="L30">
+        <v>5</v>
+      </c>
+      <c r="M30">
+        <v>50</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>396</v>
+      </c>
+      <c r="B31" t="s">
+        <v>397</v>
+      </c>
+      <c r="D31" t="s">
+        <v>514</v>
+      </c>
+      <c r="E31" t="s">
+        <v>60</v>
+      </c>
+      <c r="F31" t="s">
+        <v>44</v>
+      </c>
+      <c r="G31" t="s">
+        <v>304</v>
+      </c>
+      <c r="H31" t="s">
+        <v>299</v>
+      </c>
+      <c r="I31" t="s">
+        <v>398</v>
+      </c>
+      <c r="K31">
+        <v>30000</v>
+      </c>
+      <c r="L31">
+        <v>10</v>
+      </c>
+      <c r="M31">
+        <v>50</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>399</v>
+      </c>
+      <c r="B32" t="s">
+        <v>400</v>
+      </c>
+      <c r="D32" t="s">
+        <v>515</v>
+      </c>
+      <c r="E32" t="s">
+        <v>60</v>
+      </c>
+      <c r="F32" t="s">
+        <v>44</v>
+      </c>
+      <c r="G32" t="s">
+        <v>304</v>
+      </c>
+      <c r="H32" t="s">
+        <v>299</v>
+      </c>
+      <c r="I32" t="s">
+        <v>401</v>
+      </c>
+      <c r="K32">
+        <v>30000</v>
+      </c>
+      <c r="L32">
+        <v>25</v>
+      </c>
+      <c r="M32">
+        <v>50</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>402</v>
+      </c>
+      <c r="B33" t="s">
+        <v>403</v>
+      </c>
+      <c r="D33" t="s">
+        <v>518</v>
+      </c>
+      <c r="E33" t="s">
+        <v>60</v>
+      </c>
+      <c r="F33" t="s">
+        <v>44</v>
+      </c>
+      <c r="G33" t="s">
+        <v>304</v>
+      </c>
+      <c r="H33" t="s">
+        <v>299</v>
+      </c>
+      <c r="I33" t="s">
+        <v>404</v>
+      </c>
+      <c r="K33">
+        <v>30000</v>
+      </c>
+      <c r="L33">
+        <v>50</v>
+      </c>
+      <c r="M33">
+        <v>50</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>405</v>
+      </c>
+      <c r="B34" t="s">
+        <v>406</v>
+      </c>
+      <c r="D34" t="s">
+        <v>517</v>
+      </c>
+      <c r="E34" t="s">
+        <v>60</v>
+      </c>
+      <c r="F34" t="s">
+        <v>44</v>
+      </c>
+      <c r="G34" t="s">
+        <v>304</v>
+      </c>
+      <c r="H34" t="s">
+        <v>299</v>
+      </c>
+      <c r="I34" t="s">
+        <v>407</v>
+      </c>
+      <c r="K34">
+        <v>30000</v>
+      </c>
+      <c r="L34">
+        <v>75</v>
+      </c>
+      <c r="M34">
+        <v>50</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>408</v>
+      </c>
+      <c r="B35" t="s">
+        <v>409</v>
+      </c>
+      <c r="D35" t="s">
+        <v>522</v>
+      </c>
+      <c r="E35" t="s">
+        <v>60</v>
+      </c>
+      <c r="F35" t="s">
+        <v>44</v>
+      </c>
+      <c r="G35" t="s">
+        <v>304</v>
+      </c>
+      <c r="H35" t="s">
+        <v>299</v>
+      </c>
+      <c r="I35" t="s">
+        <v>410</v>
+      </c>
+      <c r="K35">
+        <v>30000</v>
+      </c>
+      <c r="L35">
+        <v>100</v>
+      </c>
+      <c r="M35">
+        <v>50</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>411</v>
+      </c>
+      <c r="B36" t="s">
+        <v>412</v>
+      </c>
+      <c r="D36" t="s">
+        <v>519</v>
+      </c>
+      <c r="E36" t="s">
+        <v>60</v>
+      </c>
+      <c r="F36" t="s">
+        <v>44</v>
+      </c>
+      <c r="G36" t="s">
+        <v>304</v>
+      </c>
+      <c r="H36" t="s">
+        <v>299</v>
+      </c>
+      <c r="I36" t="s">
+        <v>413</v>
+      </c>
+      <c r="K36">
+        <v>30000</v>
+      </c>
+      <c r="L36">
+        <v>150</v>
+      </c>
+      <c r="M36">
+        <v>50</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>414</v>
+      </c>
+      <c r="B37" t="s">
+        <v>415</v>
+      </c>
+      <c r="D37" t="s">
+        <v>520</v>
+      </c>
+      <c r="E37" t="s">
+        <v>60</v>
+      </c>
+      <c r="F37" t="s">
+        <v>44</v>
+      </c>
+      <c r="G37" t="s">
+        <v>304</v>
+      </c>
+      <c r="H37" t="s">
+        <v>299</v>
+      </c>
+      <c r="I37" t="s">
+        <v>416</v>
+      </c>
+      <c r="K37">
+        <v>30000</v>
+      </c>
+      <c r="L37">
+        <v>200</v>
+      </c>
+      <c r="M37">
+        <v>50</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>417</v>
+      </c>
+      <c r="B38" t="s">
+        <v>418</v>
+      </c>
+      <c r="D38" t="s">
+        <v>521</v>
+      </c>
+      <c r="E38" t="s">
+        <v>60</v>
+      </c>
+      <c r="F38" t="s">
+        <v>44</v>
+      </c>
+      <c r="G38" t="s">
+        <v>304</v>
+      </c>
+      <c r="H38" t="s">
+        <v>299</v>
+      </c>
+      <c r="I38" t="s">
+        <v>419</v>
+      </c>
+      <c r="K38">
+        <v>30000</v>
+      </c>
+      <c r="L38">
+        <v>250</v>
+      </c>
+      <c r="M38">
+        <v>50</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>420</v>
+      </c>
+      <c r="B39" t="s">
+        <v>421</v>
+      </c>
+      <c r="D39" t="s">
+        <v>516</v>
+      </c>
+      <c r="E39" t="s">
+        <v>60</v>
+      </c>
+      <c r="F39" t="s">
+        <v>44</v>
+      </c>
+      <c r="G39" t="s">
+        <v>361</v>
+      </c>
+      <c r="H39" t="s">
+        <v>299</v>
+      </c>
+      <c r="I39" t="s">
+        <v>422</v>
+      </c>
+      <c r="L39">
+        <v>5</v>
+      </c>
+      <c r="N39" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>424</v>
+      </c>
+      <c r="B40" t="s">
+        <v>425</v>
+      </c>
+      <c r="D40" t="s">
+        <v>523</v>
+      </c>
+      <c r="E40" t="s">
+        <v>60</v>
+      </c>
+      <c r="F40" t="s">
+        <v>43</v>
+      </c>
+      <c r="G40" t="s">
+        <v>304</v>
+      </c>
+      <c r="H40" t="s">
+        <v>299</v>
+      </c>
+      <c r="I40" t="s">
+        <v>426</v>
+      </c>
+      <c r="J40">
+        <v>5</v>
+      </c>
+      <c r="K40">
+        <v>30000</v>
+      </c>
+      <c r="M40">
+        <v>50</v>
+      </c>
+      <c r="Q40" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>427</v>
+      </c>
+      <c r="B41" t="s">
+        <v>428</v>
+      </c>
+      <c r="D41" t="s">
+        <v>529</v>
+      </c>
+      <c r="E41" t="s">
+        <v>60</v>
+      </c>
+      <c r="F41" t="s">
+        <v>43</v>
+      </c>
+      <c r="G41" t="s">
+        <v>304</v>
+      </c>
+      <c r="H41" t="s">
+        <v>299</v>
+      </c>
+      <c r="I41" t="s">
+        <v>429</v>
+      </c>
+      <c r="J41">
+        <v>10</v>
+      </c>
+      <c r="K41">
+        <v>30000</v>
+      </c>
+      <c r="M41">
+        <v>50</v>
+      </c>
+      <c r="Q41" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>430</v>
+      </c>
+      <c r="B42" t="s">
+        <v>431</v>
+      </c>
+      <c r="D42" t="s">
+        <v>524</v>
+      </c>
+      <c r="E42" t="s">
+        <v>60</v>
+      </c>
+      <c r="F42" t="s">
+        <v>43</v>
+      </c>
+      <c r="G42" t="s">
+        <v>304</v>
+      </c>
+      <c r="H42" t="s">
+        <v>299</v>
+      </c>
+      <c r="I42" t="s">
+        <v>432</v>
+      </c>
+      <c r="J42">
+        <v>25</v>
+      </c>
+      <c r="K42">
+        <v>30000</v>
+      </c>
+      <c r="M42">
+        <v>50</v>
+      </c>
+      <c r="Q42" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="43" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>433</v>
+      </c>
+      <c r="B43" t="s">
+        <v>434</v>
+      </c>
+      <c r="D43" t="s">
+        <v>528</v>
+      </c>
+      <c r="E43" t="s">
+        <v>60</v>
+      </c>
+      <c r="F43" t="s">
+        <v>43</v>
+      </c>
+      <c r="G43" t="s">
+        <v>304</v>
+      </c>
+      <c r="H43" t="s">
+        <v>299</v>
+      </c>
+      <c r="I43" t="s">
+        <v>435</v>
+      </c>
+      <c r="J43">
+        <v>50</v>
+      </c>
+      <c r="K43">
+        <v>30000</v>
+      </c>
+      <c r="M43">
+        <v>50</v>
+      </c>
+      <c r="Q43" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="44" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>436</v>
+      </c>
+      <c r="B44" t="s">
+        <v>437</v>
+      </c>
+      <c r="D44" t="s">
+        <v>526</v>
+      </c>
+      <c r="E44" t="s">
+        <v>60</v>
+      </c>
+      <c r="F44" t="s">
+        <v>43</v>
+      </c>
+      <c r="G44" t="s">
+        <v>304</v>
+      </c>
+      <c r="H44" t="s">
+        <v>299</v>
+      </c>
+      <c r="I44" t="s">
+        <v>438</v>
+      </c>
+      <c r="J44">
+        <v>75</v>
+      </c>
+      <c r="K44">
+        <v>30000</v>
+      </c>
+      <c r="M44">
+        <v>50</v>
+      </c>
+      <c r="Q44" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="45" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>439</v>
+      </c>
+      <c r="B45" t="s">
+        <v>440</v>
+      </c>
+      <c r="D45" t="s">
+        <v>525</v>
+      </c>
+      <c r="E45" t="s">
+        <v>60</v>
+      </c>
+      <c r="F45" t="s">
+        <v>43</v>
+      </c>
+      <c r="G45" t="s">
+        <v>304</v>
+      </c>
+      <c r="H45" t="s">
+        <v>299</v>
+      </c>
+      <c r="I45" t="s">
+        <v>441</v>
+      </c>
+      <c r="J45">
+        <v>100</v>
+      </c>
+      <c r="K45">
+        <v>30000</v>
+      </c>
+      <c r="M45">
+        <v>50</v>
+      </c>
+      <c r="Q45" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="46" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>442</v>
+      </c>
+      <c r="B46" t="s">
+        <v>443</v>
+      </c>
+      <c r="D46" t="s">
+        <v>527</v>
+      </c>
+      <c r="E46" t="s">
+        <v>60</v>
+      </c>
+      <c r="F46" t="s">
+        <v>43</v>
+      </c>
+      <c r="G46" t="s">
+        <v>361</v>
+      </c>
+      <c r="H46" t="s">
+        <v>299</v>
+      </c>
+      <c r="I46" t="s">
+        <v>444</v>
+      </c>
+      <c r="J46">
+        <v>5</v>
+      </c>
+      <c r="N46" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="47" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="B47" t="s">
+        <v>446</v>
+      </c>
+      <c r="C47" t="s">
+        <v>531</v>
+      </c>
+      <c r="E47" t="s">
+        <v>63</v>
+      </c>
+      <c r="F47" t="s">
+        <v>389</v>
+      </c>
+      <c r="G47" t="s">
+        <v>298</v>
+      </c>
+      <c r="H47" t="s">
+        <v>298</v>
+      </c>
+      <c r="I47" t="s">
+        <v>447</v>
+      </c>
+      <c r="M47" t="s">
+        <v>483</v>
+      </c>
+      <c r="Q47" t="s">
+        <v>448</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA03F59A-0EC6-450E-AE18-243FFD97199D}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="107.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="111.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>449</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>450</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>452</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>454</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>455</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>460</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>455</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>463</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC46E614-3935-4A35-AF14-2BF587B575D4}">
+  <dimension ref="A1:B24"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="30.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="84.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>464</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>466</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>468</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B4" s="10"/>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>470</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>287</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>288</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>289</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>290</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>291</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>479</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>295</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>296</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B24" s="12"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{599491C1-ECFA-4332-92BD-67AB5ED41907}">
   <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>